<commit_message>
feat: complete AI analytics platform
</commit_message>
<xml_diff>
--- a/backend/app/exports/reviews.xlsx
+++ b/backend/app/exports/reviews.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,16 +455,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>renkeri berbattı</t>
+          <t>ürün beklediğim kadar iyi değildi kumaşı çok kalın tavsiye etmiyorum</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The customer is highly dissatisfied with the color of the product.</t>
+          <t>The customer is dissatisfied with the product's quality and the thickness of the fabric, leading to a negative recommendation.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,115 +479,185 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>['Product Quality', 'Design']</t>
+          <t>['Product Quality', 'Apparel']</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>['color', 'terrible', 'appearance']</t>
+          <t>['ürün kalitesi', 'kumaş kalınlığı', 'tavsiye etmiyorum', 'beklenti']</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ürünüç ok beğendim ama yanlış renk geldi</t>
+          <t>ürünü çok beğendim ve çok hızlı geldi kesinlikle tekrar buradan alışveriş yapacağım</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The customer is satisfied with the product quality but received the item in the wrong color.</t>
+          <t>The customer is highly satisfied with both the product quality and the fast delivery service.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Disappointment</t>
+          <t>Joy</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>['Product Quality', 'Logistics', 'Order Fulfillment']</t>
+          <t>['Product Quality', 'Shipping and Delivery', 'Customer Satisfaction']</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>['ürün', 'yanlış renk', 'teslimat', 'sipariş']</t>
+          <t>['ürün beğenisi', 'hızlı teslimat', 'tekrar alışveriş']</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ürünü çok beğendim</t>
+          <t>renkeri berbattı</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>The customer expressed that they liked the product very much.</t>
+          <t>The customer is highly dissatisfied with the color of the product.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Joy</t>
+          <t>Disappointment</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>['Product Satisfaction', 'Retail']</t>
+          <t>['Product Quality', 'Design']</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>['ürün', 'beğendim', 'memnuniyet']</t>
+          <t>['color', 'terrible', 'appearance']</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ürünüç ok beğendim ama yanlış renk geldi</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The customer is satisfied with the product quality but received the item in the wrong color.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Disappointment</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>['Product Quality', 'Logistics', 'Order Fulfillment']</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>['ürün', 'yanlış renk', 'teslimat', 'sipariş']</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ürünü çok beğendim</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The customer expressed that they liked the product very much.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Joy</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>['Product Satisfaction', 'Retail']</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>['ürün', 'beğendim', 'memnuniyet']</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
         <v>1</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>ürün baya kötü</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>The customer is highly dissatisfied, stating that the product is very poor.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Disappointment</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>['Product Quality']</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>['ürün', 'kötü', 'kalite']</t>
         </is>

</xml_diff>